<commit_message>
Fix règle de gestion b923ce31cc30fe4693a22510f556b41559e233c1
</commit_message>
<xml_diff>
--- a/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/CodeSystem-tddui-discriminator.xlsx
+++ b/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/CodeSystem-tddui-discriminator.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-16T10:03:26+00:00</t>
+    <t>2026-06-16T13:10:49+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -78,7 +78,7 @@
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t>France</t>
+    <t>France (la)</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>